<commit_message>
adding tables and stuff
</commit_message>
<xml_diff>
--- a/results/Supplementary_Table_1_SpiderAccessions_BUSCOs.xlsx
+++ b/results/Supplementary_Table_1_SpiderAccessions_BUSCOs.xlsx
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Acroaspis_sp_IDV6688</t>
+          <t>Argiope_bruennichi</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -482,24 +482,24 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2280</v>
+        <v>2354</v>
       </c>
       <c r="E2" t="n">
-        <v>429</v>
+        <v>374</v>
       </c>
       <c r="F2" t="n">
-        <v>2709</v>
+        <v>2728</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>IANO01</t>
+          <t>IBFJ01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Acrosomoides_sp_IDV7426</t>
+          <t>Argiope_aetheroides</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -513,24 +513,24 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2306</v>
+        <v>2344</v>
       </c>
       <c r="E3" t="n">
-        <v>338</v>
+        <v>375</v>
       </c>
       <c r="F3" t="n">
-        <v>2644</v>
+        <v>2719</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>ICOJ01</t>
+          <t>IASB01</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ainerigone_saitoi</t>
+          <t>Caerostris_darwini</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -540,28 +540,28 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2238</v>
+        <v>2337</v>
       </c>
       <c r="E4" t="n">
-        <v>550</v>
+        <v>358</v>
       </c>
       <c r="F4" t="n">
-        <v>2788</v>
+        <v>2695</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>IBTE01</t>
+          <t>ICOF01</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ambicodamus_IDV6680</t>
+          <t>Argiope_keyserlingi</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -571,59 +571,59 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Nicodamidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2261</v>
+        <v>2324</v>
       </c>
       <c r="E5" t="n">
-        <v>409</v>
+        <v>394</v>
       </c>
       <c r="F5" t="n">
-        <v>2670</v>
+        <v>2718</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ICBW01</t>
+          <t>IAET01</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Antrodiaetus_roretzi</t>
+          <t>Eriophora_pustulosa</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mygalomorphae</t>
+          <t>Araneomorphae</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Antrodiaetidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2190</v>
+        <v>2321</v>
       </c>
       <c r="E6" t="n">
-        <v>349</v>
+        <v>421</v>
       </c>
       <c r="F6" t="n">
-        <v>2539</v>
+        <v>2742</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>IBPI01</t>
+          <t>IBIK01</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Araneus_inustus</t>
+          <t>Caerostris_extrusa</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -637,24 +637,24 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2261</v>
+        <v>2319</v>
       </c>
       <c r="E7" t="n">
-        <v>385</v>
+        <v>336</v>
       </c>
       <c r="F7" t="n">
-        <v>2646</v>
+        <v>2655</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>IAHS01</t>
+          <t>ICOE01</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Arcuphantes_paiki</t>
+          <t>Backobourkia_brouni</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -664,28 +664,28 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2217</v>
+        <v>2313</v>
       </c>
       <c r="E8" t="n">
-        <v>483</v>
+        <v>342</v>
       </c>
       <c r="F8" t="n">
-        <v>2700</v>
+        <v>2655</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IAWN01</t>
+          <t>ICCG01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Arcuphantes_tamaensis</t>
+          <t>Acrosomoides_sp_IDV7426</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -695,28 +695,28 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2326</v>
+        <v>2306</v>
       </c>
       <c r="E9" t="n">
-        <v>433</v>
+        <v>338</v>
       </c>
       <c r="F9" t="n">
-        <v>2759</v>
+        <v>2644</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>IAKU01</t>
+          <t>ICOJ01</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Arcuphantes_uenoi</t>
+          <t>Poecilopachys_australasia</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -726,28 +726,28 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2330</v>
+        <v>2306</v>
       </c>
       <c r="E10" t="n">
-        <v>488</v>
+        <v>388</v>
       </c>
       <c r="F10" t="n">
-        <v>2818</v>
+        <v>2694</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>IBBK01</t>
+          <t>ICKB01</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Argiope_aetheroides</t>
+          <t>Dolophones_sp_IDV6683</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -761,24 +761,24 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2344</v>
+        <v>2304</v>
       </c>
       <c r="E11" t="n">
-        <v>375</v>
+        <v>440</v>
       </c>
       <c r="F11" t="n">
-        <v>2719</v>
+        <v>2744</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>IASB01</t>
+          <t>IBZG01</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Argiope_bruennichi</t>
+          <t>Phonognatha_graeffei</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -792,24 +792,24 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2354</v>
+        <v>2301</v>
       </c>
       <c r="E12" t="n">
-        <v>374</v>
+        <v>359</v>
       </c>
       <c r="F12" t="n">
-        <v>2728</v>
+        <v>2660</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>IBFJ01</t>
+          <t>IATW01</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Argiope_keyserlingi</t>
+          <t>Lariniaria_argiopiformis</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -823,24 +823,24 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2324</v>
+        <v>2296</v>
       </c>
       <c r="E13" t="n">
-        <v>394</v>
+        <v>372</v>
       </c>
       <c r="F13" t="n">
-        <v>2718</v>
+        <v>2668</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>IAET01</t>
+          <t>IAFI01</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Argyrodes_flavescens</t>
+          <t>Hypsosinga_pygmaea</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -850,28 +850,28 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Theridiidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2294</v>
+        <v>2283</v>
       </c>
       <c r="E14" t="n">
-        <v>353</v>
+        <v>443</v>
       </c>
       <c r="F14" t="n">
-        <v>2647</v>
+        <v>2726</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>IAFU01</t>
+          <t>ICEG01</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Argyrodes_miniaceus</t>
+          <t>Acroaspis_sp_IDV6688</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -881,28 +881,28 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Theridiidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2226</v>
+        <v>2280</v>
       </c>
       <c r="E15" t="n">
-        <v>417</v>
+        <v>429</v>
       </c>
       <c r="F15" t="n">
-        <v>2643</v>
+        <v>2709</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>IBQT01</t>
+          <t>IANO01</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Backobourkia_brouni</t>
+          <t>Neoscona_subpullata</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -916,24 +916,24 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2313</v>
+        <v>2280</v>
       </c>
       <c r="E16" t="n">
-        <v>342</v>
+        <v>472</v>
       </c>
       <c r="F16" t="n">
-        <v>2655</v>
+        <v>2752</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>ICCG01</t>
+          <t>IBPZ01</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Baryphymula_kamakuraensis</t>
+          <t>Plebs_sachalinensis</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -943,28 +943,28 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2236</v>
+        <v>2273</v>
       </c>
       <c r="E17" t="n">
-        <v>582</v>
+        <v>403</v>
       </c>
       <c r="F17" t="n">
-        <v>2818</v>
+        <v>2676</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>IBGF01</t>
+          <t>ICHT01</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Caerostris_darwini</t>
+          <t>Larinioides_cornutus</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -978,24 +978,24 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2337</v>
+        <v>2271</v>
       </c>
       <c r="E18" t="n">
-        <v>358</v>
+        <v>393</v>
       </c>
       <c r="F18" t="n">
-        <v>2695</v>
+        <v>2664</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>ICOF01, GGTX01</t>
+          <t>IAHZ01</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Caerostris_extrusa</t>
+          <t>Metazygia_zilloides</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1009,24 +1009,24 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2319</v>
+        <v>2270</v>
       </c>
       <c r="E19" t="n">
-        <v>336</v>
+        <v>414</v>
       </c>
       <c r="F19" t="n">
-        <v>2655</v>
+        <v>2684</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>ICOE01</t>
+          <t>IBDY01</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Chrysso_octomaculata</t>
+          <t>Neoscona_theisi</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1036,28 +1036,28 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Theridiidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2212</v>
+        <v>2268</v>
       </c>
       <c r="E20" t="n">
-        <v>537</v>
+        <v>398</v>
       </c>
       <c r="F20" t="n">
-        <v>2749</v>
+        <v>2666</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>IBWR01</t>
+          <t>IAXT01</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Clubiona_robusta</t>
+          <t>Cyclosa_octotuberculata</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1067,28 +1067,28 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Clubionidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2248</v>
+        <v>2267</v>
       </c>
       <c r="E21" t="n">
-        <v>417</v>
+        <v>381</v>
       </c>
       <c r="F21" t="n">
-        <v>2665</v>
+        <v>2648</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ICJS01</t>
+          <t>IAQZ01</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cryptachaea_gigantipes</t>
+          <t>Larinia_phthisica</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1098,28 +1098,28 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Theridiidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>2266</v>
+        <v>2265</v>
       </c>
       <c r="E22" t="n">
-        <v>396</v>
+        <v>432</v>
       </c>
       <c r="F22" t="n">
-        <v>2662</v>
+        <v>2697</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>IBTR01</t>
+          <t>IAJV01</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cyclosa_octotuberculata</t>
+          <t>Cyrtophora_cicatrosa</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1133,24 +1133,24 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2267</v>
+        <v>2262</v>
       </c>
       <c r="E23" t="n">
-        <v>381</v>
+        <v>402</v>
       </c>
       <c r="F23" t="n">
-        <v>2648</v>
+        <v>2664</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>IAQZ01</t>
+          <t>IBHY01</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Cyrtarachne_bufo</t>
+          <t>Araneus_inustus</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1164,24 +1164,24 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>2254</v>
+        <v>2261</v>
       </c>
       <c r="E24" t="n">
-        <v>440</v>
+        <v>385</v>
       </c>
       <c r="F24" t="n">
-        <v>2694</v>
+        <v>2646</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>ICFD01</t>
+          <t>IAHS01</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cyrtophora_cicatrosa</t>
+          <t>Neoscona_scylla</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1195,24 +1195,24 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2262</v>
+        <v>2257</v>
       </c>
       <c r="E25" t="n">
-        <v>402</v>
+        <v>413</v>
       </c>
       <c r="F25" t="n">
-        <v>2664</v>
+        <v>2670</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>IBHY01</t>
+          <t>IAEU01</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Deinopis_sp_IDV6783</t>
+          <t>Neoscona_adianta</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1222,28 +1222,28 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Deinopidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>2203</v>
+        <v>2256</v>
       </c>
       <c r="E26" t="n">
-        <v>433</v>
+        <v>407</v>
       </c>
       <c r="F26" t="n">
-        <v>2636</v>
+        <v>2663</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>IBBP01</t>
+          <t>IBRX01</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Deinopis_sp_IDV7365</t>
+          <t>Cyrtarachne_bufo</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1253,28 +1253,28 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Deinopidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2209</v>
+        <v>2254</v>
       </c>
       <c r="E27" t="n">
-        <v>395</v>
+        <v>440</v>
       </c>
       <c r="F27" t="n">
-        <v>2604</v>
+        <v>2694</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>ICOI01</t>
+          <t>ICFD01</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Desis_marina</t>
+          <t>Neoscona_nautica</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1284,28 +1284,28 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Desidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2063</v>
+        <v>2254</v>
       </c>
       <c r="E28" t="n">
-        <v>624</v>
+        <v>520</v>
       </c>
       <c r="F28" t="n">
-        <v>2687</v>
+        <v>2774</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>GIWQ01</t>
+          <t>ICBF01</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Diaea_subdola</t>
+          <t>Nuctenea_umbratica</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1315,28 +1315,28 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Thomisidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2281</v>
+        <v>2248</v>
       </c>
       <c r="E29" t="n">
-        <v>416</v>
+        <v>442</v>
       </c>
       <c r="F29" t="n">
-        <v>2697</v>
+        <v>2690</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>ICGF01</t>
+          <t>IAPM01</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Doenitzius_peniculus</t>
+          <t>Ordgarius_hobsoni</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1346,28 +1346,28 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2330</v>
+        <v>2219</v>
       </c>
       <c r="E30" t="n">
-        <v>467</v>
+        <v>438</v>
       </c>
       <c r="F30" t="n">
-        <v>2797</v>
+        <v>2657</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>IBJ01</t>
+          <t>IAGL01</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Doenitzius_pruvus</t>
+          <t>Ordgarius_sexspinosus</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1377,28 +1377,28 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Araneidae</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2285</v>
+        <v>2188</v>
       </c>
       <c r="E31" t="n">
-        <v>551</v>
+        <v>455</v>
       </c>
       <c r="F31" t="n">
-        <v>2836</v>
+        <v>2643</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>IBVW01</t>
+          <t>ICMU01</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Dolophones_sp_IDV6683</t>
+          <t>Clubiona_robusta</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1408,28 +1408,28 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Clubionidae</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2304</v>
+        <v>2248</v>
       </c>
       <c r="E32" t="n">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="F32" t="n">
-        <v>2744</v>
+        <v>2665</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>IBZG01</t>
+          <t>ICJS01</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Drapetisca_socialis</t>
+          <t>Phrurolithus_coreanus</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1439,28 +1439,28 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Corinnidae</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2206</v>
+        <v>2116</v>
       </c>
       <c r="E33" t="n">
-        <v>582</v>
+        <v>683</v>
       </c>
       <c r="F33" t="n">
-        <v>2788</v>
+        <v>2799</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>ICKS01</t>
+          <t>IBPN01</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ebrechtella_tricuspidata</t>
+          <t>Deinopis_sp_IDV7365</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1470,28 +1470,28 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Thomisidae</t>
+          <t>Deinopidae</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>2256</v>
+        <v>2209</v>
       </c>
       <c r="E34" t="n">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="F34" t="n">
-        <v>2645</v>
+        <v>2604</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>ICBZ01</t>
+          <t>ICOI01</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Eriophora_pustulosa</t>
+          <t>Deinopis_sp_IDV6783</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1501,28 +1501,28 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Deinopidae</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>2321</v>
+        <v>2203</v>
       </c>
       <c r="E35" t="n">
-        <v>421</v>
+        <v>433</v>
       </c>
       <c r="F35" t="n">
-        <v>2742</v>
+        <v>2636</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>IBIK01</t>
+          <t>IBBP01</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Falcileptoneta_japonica</t>
+          <t>Desis_marina</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1532,28 +1532,28 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Leptonetidae</t>
+          <t>Desidae</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>2339</v>
+        <v>2063</v>
       </c>
       <c r="E36" t="n">
-        <v>431</v>
+        <v>624</v>
       </c>
       <c r="F36" t="n">
-        <v>2770</v>
+        <v>2687</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>ICFE01</t>
+          <t>GIWQ01</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Floronia_bucculenta</t>
+          <t>Paratheuma_awasensis</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1563,28 +1563,28 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Dictynidae</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>2250</v>
+        <v>2215</v>
       </c>
       <c r="E37" t="n">
-        <v>464</v>
+        <v>437</v>
       </c>
       <c r="F37" t="n">
-        <v>2714</v>
+        <v>2652</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>ICGA01</t>
+          <t>IARK01</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Gnathonarium_exsiccatum</t>
+          <t>Zelotes_iriomotensis</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1594,24 +1594,28 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Gnaphosidae</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>2185</v>
+        <v>2214</v>
       </c>
       <c r="E38" t="n">
-        <v>580</v>
+        <v>514</v>
       </c>
       <c r="F38" t="n">
-        <v>2765</v>
-      </c>
-      <c r="G38" t="inlineStr"/>
+        <v>2728</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>IAHP01</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Helpis_minitabunda</t>
+          <t>Neoantistea_quelpartensis</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1621,28 +1625,28 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Salticidae</t>
+          <t>Hahniidae</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>2238</v>
+        <v>2299</v>
       </c>
       <c r="E39" t="n">
-        <v>405</v>
+        <v>393</v>
       </c>
       <c r="F39" t="n">
-        <v>2643</v>
+        <v>2692</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>IAUM01</t>
+          <t>IBHE01</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Hypselistes_asiaticus</t>
+          <t>Masirana_silvicola</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1652,28 +1656,28 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Leptonetidae</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2217</v>
+        <v>2371</v>
       </c>
       <c r="E40" t="n">
-        <v>546</v>
+        <v>399</v>
       </c>
       <c r="F40" t="n">
-        <v>2763</v>
+        <v>2770</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>IAOT01</t>
+          <t>ICEN01</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Hypsosinga_pygmaea</t>
+          <t>Falcileptoneta_japonica</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1683,28 +1687,28 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Leptonetidae</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>2283</v>
+        <v>2339</v>
       </c>
       <c r="E41" t="n">
-        <v>443</v>
+        <v>431</v>
       </c>
       <c r="F41" t="n">
-        <v>2726</v>
+        <v>2770</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>ICEG01</t>
+          <t>ICFE01</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Larinia_phthisica</t>
+          <t>Ryojius_japonicus</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1714,28 +1718,28 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2265</v>
+        <v>2368</v>
       </c>
       <c r="E42" t="n">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="F42" t="n">
-        <v>2697</v>
+        <v>2801</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>IAJV01</t>
+          <t>IBWO01</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Lariniaria_argiopiformis</t>
+          <t>Syedra_oii</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1745,28 +1749,28 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2296</v>
+        <v>2355</v>
       </c>
       <c r="E43" t="n">
-        <v>372</v>
+        <v>405</v>
       </c>
       <c r="F43" t="n">
-        <v>2668</v>
+        <v>2760</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>IAFI01</t>
+          <t>IAXS01</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Larinioides_cornutus</t>
+          <t>Arcuphantes_uenoi</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1776,28 +1780,28 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2271</v>
+        <v>2330</v>
       </c>
       <c r="E44" t="n">
-        <v>393</v>
+        <v>488</v>
       </c>
       <c r="F44" t="n">
-        <v>2664</v>
+        <v>2818</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>IAHZ01</t>
+          <t>IBBK01</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Latrodectus_hasseltii</t>
+          <t>Doenitzius_peniculus</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1807,28 +1811,28 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Theridiidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>2249</v>
+        <v>2330</v>
       </c>
       <c r="E45" t="n">
-        <v>431</v>
+        <v>467</v>
       </c>
       <c r="F45" t="n">
-        <v>2680</v>
+        <v>2797</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>IBKS01</t>
+          <t>IBJ01</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Lehtinelagia_evanida</t>
+          <t>Arcuphantes_tamaensis</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1838,28 +1842,28 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Thomisidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2319</v>
+        <v>2326</v>
       </c>
       <c r="E46" t="n">
-        <v>324</v>
+        <v>433</v>
       </c>
       <c r="F46" t="n">
-        <v>2643</v>
+        <v>2759</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>IBFM01</t>
+          <t>IAKU01</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Leucauge_dromedari</t>
+          <t>Saaristoa_nipponica</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1869,28 +1873,28 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>2284</v>
+        <v>2304</v>
       </c>
       <c r="E47" t="n">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="F47" t="n">
-        <v>2740</v>
+        <v>2755</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>IBHV01</t>
+          <t>IBAR01</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Masirana_silvicola</t>
+          <t>Saitonia_ojiroensis</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1900,28 +1904,28 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Leptonetidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>2371</v>
+        <v>2289</v>
       </c>
       <c r="E48" t="n">
-        <v>399</v>
+        <v>466</v>
       </c>
       <c r="F48" t="n">
-        <v>2770</v>
+        <v>2755</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>ICEN01</t>
+          <t>IAHB01</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Mesida_sp_IDV5268</t>
+          <t>Doenitzius_pruvus</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1931,24 +1935,28 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>2310</v>
+        <v>2285</v>
       </c>
       <c r="E49" t="n">
-        <v>421</v>
+        <v>551</v>
       </c>
       <c r="F49" t="n">
-        <v>2731</v>
-      </c>
-      <c r="G49" t="inlineStr"/>
+        <v>2836</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>IBVW01</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Metazygia_zilloides</t>
+          <t>Neriene_oidedicata</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1958,28 +1966,28 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>2270</v>
+        <v>2271</v>
       </c>
       <c r="E50" t="n">
-        <v>414</v>
+        <v>394</v>
       </c>
       <c r="F50" t="n">
-        <v>2684</v>
+        <v>2665</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>IBDY01</t>
+          <t>IAQC01</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Metleucauge_yunohamensis</t>
+          <t>Microbathyphantes_tateyamaensis</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1989,28 +1997,28 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2229</v>
+        <v>2253</v>
       </c>
       <c r="E51" t="n">
-        <v>441</v>
+        <v>542</v>
       </c>
       <c r="F51" t="n">
-        <v>2670</v>
+        <v>2795</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>IBVS01</t>
+          <t>ICFH01</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Microbathyphantes_tateyamaensis</t>
+          <t>Floronia_bucculenta</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2024,24 +2032,24 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2253</v>
+        <v>2250</v>
       </c>
       <c r="E52" t="n">
-        <v>542</v>
+        <v>464</v>
       </c>
       <c r="F52" t="n">
-        <v>2795</v>
+        <v>2714</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>ICFH01</t>
+          <t>ICGA01</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Neoantistea_quelpartensis</t>
+          <t>Ainerigone_saitoi</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2051,28 +2059,28 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Hahniidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>2299</v>
+        <v>2238</v>
       </c>
       <c r="E53" t="n">
-        <v>393</v>
+        <v>550</v>
       </c>
       <c r="F53" t="n">
-        <v>2692</v>
+        <v>2788</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>IBHE01</t>
+          <t>IBTE01</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Neon_minutus</t>
+          <t>Baryphymula_kamakuraensis</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2082,28 +2090,28 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Salticidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>2309</v>
+        <v>2236</v>
       </c>
       <c r="E54" t="n">
-        <v>490</v>
+        <v>582</v>
       </c>
       <c r="F54" t="n">
-        <v>2799</v>
+        <v>2818</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>IAIC01</t>
+          <t>IBGF01</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Neoscona_adianta</t>
+          <t>Arcuphantes_paiki</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2113,28 +2121,28 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>2256</v>
+        <v>2217</v>
       </c>
       <c r="E55" t="n">
-        <v>407</v>
+        <v>483</v>
       </c>
       <c r="F55" t="n">
-        <v>2663</v>
+        <v>2700</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>IBRX01</t>
+          <t>IAWN01</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Neoscona_nautica</t>
+          <t>Hypselistes_asiaticus</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2144,28 +2152,28 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>2254</v>
+        <v>2217</v>
       </c>
       <c r="E56" t="n">
-        <v>520</v>
+        <v>546</v>
       </c>
       <c r="F56" t="n">
-        <v>2774</v>
+        <v>2763</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>ICBF01</t>
+          <t>IAOT01</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Neoscona_scylla</t>
+          <t>Ummeliata_osakaensis</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2175,28 +2183,28 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>2257</v>
+        <v>2214</v>
       </c>
       <c r="E57" t="n">
-        <v>413</v>
+        <v>552</v>
       </c>
       <c r="F57" t="n">
-        <v>2670</v>
+        <v>2766</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>IAEU01</t>
+          <t>IBXZ01</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Neoscona_subpullata</t>
+          <t>Drapetisca_socialis</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2206,28 +2214,28 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>2280</v>
+        <v>2206</v>
       </c>
       <c r="E58" t="n">
-        <v>472</v>
+        <v>582</v>
       </c>
       <c r="F58" t="n">
-        <v>2752</v>
+        <v>2788</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>IBPZ01</t>
+          <t>ICKS01</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Neoscona_theisi</t>
+          <t>Gnathonarium_exsiccatum</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2237,21 +2245,21 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Linyphiidae</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>2268</v>
+        <v>2185</v>
       </c>
       <c r="E59" t="n">
-        <v>398</v>
+        <v>580</v>
       </c>
       <c r="F59" t="n">
-        <v>2666</v>
+        <v>2765</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>IAXT01</t>
+          <t>ICCR01</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2297,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Neriene_oidedicata</t>
+          <t>Pseudomicrargus_latitegulatus</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2303,24 +2311,24 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>2271</v>
+        <v>2116</v>
       </c>
       <c r="E61" t="n">
-        <v>394</v>
+        <v>690</v>
       </c>
       <c r="F61" t="n">
-        <v>2665</v>
+        <v>2806</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>IAQC01</t>
+          <t>IBJR01</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Nuctenea_umbratica</t>
+          <t>Pardosa_graminea</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2330,28 +2338,28 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Lycosidae</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>2248</v>
+        <v>2277</v>
       </c>
       <c r="E62" t="n">
-        <v>442</v>
+        <v>425</v>
       </c>
       <c r="F62" t="n">
-        <v>2690</v>
+        <v>2702</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>IAPM01</t>
+          <t>ICDS01</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Orchestina_okitsui</t>
+          <t>Piratula_tanakai</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2361,28 +2369,28 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Oonopidae</t>
+          <t>Lycosidae</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>2101</v>
+        <v>2245</v>
       </c>
       <c r="E63" t="n">
-        <v>548</v>
+        <v>472</v>
       </c>
       <c r="F63" t="n">
-        <v>2649</v>
+        <v>2717</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>IAOP01</t>
+          <t>IBYA01</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Ordgarius_hobsoni</t>
+          <t>Ambicodamus_IDV6680</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2392,28 +2400,28 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Nicodamidae</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>2219</v>
+        <v>2261</v>
       </c>
       <c r="E64" t="n">
-        <v>438</v>
+        <v>409</v>
       </c>
       <c r="F64" t="n">
-        <v>2657</v>
+        <v>2670</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>IAGL01</t>
+          <t>ICBW01</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Ordgarius_sexspinosus</t>
+          <t>Orchestina_okitsui</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2423,28 +2431,28 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Oonopidae</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>2188</v>
+        <v>2101</v>
       </c>
       <c r="E65" t="n">
-        <v>455</v>
+        <v>548</v>
       </c>
       <c r="F65" t="n">
-        <v>2643</v>
+        <v>2649</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>ICMU01</t>
+          <t>IAOP01</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Oxytate_striatipes</t>
+          <t>Psechrus_IDV5238</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2454,28 +2462,28 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Thomisidae</t>
+          <t>Psechridae</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>2242</v>
+        <v>2281</v>
       </c>
       <c r="E66" t="n">
-        <v>483</v>
+        <v>405</v>
       </c>
       <c r="F66" t="n">
-        <v>2725</v>
+        <v>2686</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>IALM01</t>
+          <t>IAQN01</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Ozyptila_nongae</t>
+          <t>Neon_minutus</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2485,28 +2493,28 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Thomisidae</t>
+          <t>Salticidae</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>2177</v>
+        <v>2309</v>
       </c>
       <c r="E67" t="n">
-        <v>536</v>
+        <v>490</v>
       </c>
       <c r="F67" t="n">
-        <v>2713</v>
+        <v>2799</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>ICBR01</t>
+          <t>IAIC01</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Parasteatoda_culicivora</t>
+          <t>Helpis_minitabunda</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2516,28 +2524,28 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Theridiidae</t>
+          <t>Salticidae</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>2204</v>
+        <v>2238</v>
       </c>
       <c r="E68" t="n">
-        <v>439</v>
+        <v>405</v>
       </c>
       <c r="F68" t="n">
         <v>2643</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>IBTW01</t>
+          <t>IAUM01</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Paratheuma_awasensis</t>
+          <t>Stertinius_kumadai</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2547,28 +2555,28 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Dictynidae</t>
+          <t>Salticidae</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>2215</v>
+        <v>2217</v>
       </c>
       <c r="E69" t="n">
-        <v>437</v>
+        <v>511</v>
       </c>
       <c r="F69" t="n">
-        <v>2652</v>
+        <v>2728</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>IARK01</t>
+          <t>IAUC01</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Pardosa_graminea</t>
+          <t>Mesida_sp_IDV5268</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2578,28 +2586,28 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Lycosidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>2277</v>
+        <v>2310</v>
       </c>
       <c r="E70" t="n">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="F70" t="n">
-        <v>2702</v>
+        <v>2731</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>ICDS01</t>
+          <t>ICDG01</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Pharta_brevipalpus</t>
+          <t>Leucauge_dromedari</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2609,28 +2617,28 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Thomisidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="E71" t="n">
-        <v>388</v>
+        <v>456</v>
       </c>
       <c r="F71" t="n">
-        <v>2669</v>
+        <v>2740</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>IAWA01</t>
+          <t>IBHV01</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Phonognatha_graeffei</t>
+          <t>Tetragnatha_vermiformis</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2640,28 +2648,28 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>2301</v>
+        <v>2267</v>
       </c>
       <c r="E72" t="n">
-        <v>359</v>
+        <v>374</v>
       </c>
       <c r="F72" t="n">
-        <v>2660</v>
+        <v>2641</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>IATW01</t>
+          <t>IAJJ01</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Phrurolithus_coreanus</t>
+          <t>Tetragnatha_waikamoi</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2671,28 +2679,28 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Corinnidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>2116</v>
+        <v>2266</v>
       </c>
       <c r="E73" t="n">
-        <v>683</v>
+        <v>527</v>
       </c>
       <c r="F73" t="n">
-        <v>2799</v>
+        <v>2793</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>IBPN01</t>
+          <t>GITR01</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Piratula_tanakai</t>
+          <t>Tetragnatha_paludicola</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2702,28 +2710,28 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Lycosidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2245</v>
+        <v>2260</v>
       </c>
       <c r="E74" t="n">
-        <v>472</v>
+        <v>544</v>
       </c>
       <c r="F74" t="n">
-        <v>2717</v>
+        <v>2804</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>IBYA01</t>
+          <t>GITO01</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Plebs_sachalinensis</t>
+          <t>Tetragnatha_quasimodo</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2733,28 +2741,28 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2273</v>
+        <v>2258</v>
       </c>
       <c r="E75" t="n">
-        <v>403</v>
+        <v>534</v>
       </c>
       <c r="F75" t="n">
-        <v>2676</v>
+        <v>2792</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>ICHT01</t>
+          <t>GITP01</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Poecilopachys_australasia</t>
+          <t>Tetragnatha_filiciphilia</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2764,28 +2772,28 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Araneidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>2306</v>
+        <v>2257</v>
       </c>
       <c r="E76" t="n">
-        <v>388</v>
+        <v>499</v>
       </c>
       <c r="F76" t="n">
-        <v>2694</v>
+        <v>2756</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>ICKB01</t>
+          <t>GITN01</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Psechrus_IDV5238</t>
+          <t>Tetragnatha_mandibulata</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2795,28 +2803,28 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Psechridae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>2281</v>
+        <v>2231</v>
       </c>
       <c r="E77" t="n">
-        <v>405</v>
+        <v>470</v>
       </c>
       <c r="F77" t="n">
-        <v>2686</v>
+        <v>2701</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>IAQN01</t>
+          <t>ICFC01</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Pseudomicrargus_latitegulatus</t>
+          <t>Metleucauge_yunohamensis</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2826,24 +2834,28 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>2116</v>
+        <v>2229</v>
       </c>
       <c r="E78" t="n">
-        <v>690</v>
+        <v>441</v>
       </c>
       <c r="F78" t="n">
-        <v>2806</v>
-      </c>
-      <c r="G78" t="inlineStr"/>
+        <v>2670</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>IBVS01</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Rhomphaea_labiata</t>
+          <t>Tetragnatha_stelarobusta</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2853,28 +2865,28 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Theridiidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>2249</v>
+        <v>2226</v>
       </c>
       <c r="E79" t="n">
-        <v>427</v>
+        <v>565</v>
       </c>
       <c r="F79" t="n">
-        <v>2676</v>
+        <v>2791</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>ICFA01</t>
+          <t>GITQ01</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Robertus_nojimai</t>
+          <t>Tetragnatha_brevignatha</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2884,28 +2896,28 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Theridiidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>2335</v>
+        <v>2221</v>
       </c>
       <c r="E80" t="n">
-        <v>442</v>
+        <v>583</v>
       </c>
       <c r="F80" t="n">
-        <v>2777</v>
+        <v>2804</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>ICAL01</t>
+          <t>GITM01</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Ryojius_japonicus</t>
+          <t>Tetragnatha_maxillosa</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2915,24 +2927,28 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>2368</v>
+        <v>2199</v>
       </c>
       <c r="E81" t="n">
-        <v>433</v>
+        <v>448</v>
       </c>
       <c r="F81" t="n">
-        <v>2801</v>
-      </c>
-      <c r="G81" t="inlineStr"/>
+        <v>2647</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>ICMP01</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Saaristoa_nipponica</t>
+          <t>Tetragnatha_yesoensis</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2942,24 +2958,28 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>2304</v>
+        <v>2184</v>
       </c>
       <c r="E82" t="n">
-        <v>451</v>
+        <v>508</v>
       </c>
       <c r="F82" t="n">
-        <v>2755</v>
-      </c>
-      <c r="G82" t="inlineStr"/>
+        <v>2692</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>IBMZ01</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Saitonia_ojiroensis</t>
+          <t>Tetragnatha_extensa</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2969,24 +2989,28 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Tetragnathidae</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>2289</v>
+        <v>2164</v>
       </c>
       <c r="E83" t="n">
-        <v>466</v>
+        <v>484</v>
       </c>
       <c r="F83" t="n">
-        <v>2755</v>
-      </c>
-      <c r="G83" t="inlineStr"/>
+        <v>2648</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>IAHF01</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Steatoda_grossa</t>
+          <t>Robertus_nojimai</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3000,24 +3024,24 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>2304</v>
+        <v>2335</v>
       </c>
       <c r="E84" t="n">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="F84" t="n">
-        <v>2745</v>
+        <v>2777</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>IAPP01</t>
+          <t>ICAL01</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Stephanopis_cambridgei</t>
+          <t>Steatoda_grossa</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3027,28 +3051,28 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Thomisidae</t>
+          <t>Theridiidae</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>2235</v>
+        <v>2304</v>
       </c>
       <c r="E85" t="n">
-        <v>416</v>
+        <v>441</v>
       </c>
       <c r="F85" t="n">
-        <v>2651</v>
+        <v>2745</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>ICHM01</t>
+          <t>IAPP01</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Stertinius_kumadai</t>
+          <t>Argyrodes_flavescens</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -3058,28 +3082,28 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Salticidae</t>
+          <t>Theridiidae</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>2217</v>
+        <v>2294</v>
       </c>
       <c r="E86" t="n">
-        <v>511</v>
+        <v>353</v>
       </c>
       <c r="F86" t="n">
-        <v>2728</v>
+        <v>2647</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>IAUC01</t>
+          <t>IAFU01</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Syedra_oii</t>
+          <t>Cryptachaea_gigantipes</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3089,19 +3113,23 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Theridiidae</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>2355</v>
+        <v>2266</v>
       </c>
       <c r="E87" t="n">
-        <v>405</v>
+        <v>396</v>
       </c>
       <c r="F87" t="n">
-        <v>2760</v>
-      </c>
-      <c r="G87" t="inlineStr"/>
+        <v>2662</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>IBTR01</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3137,7 +3165,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Tetragnatha_brevignatha</t>
+          <t>Latrodectus_hasseltii</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -3147,28 +3175,28 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Theridiidae</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>2221</v>
+        <v>2249</v>
       </c>
       <c r="E89" t="n">
-        <v>583</v>
+        <v>431</v>
       </c>
       <c r="F89" t="n">
-        <v>2804</v>
+        <v>2680</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>GITM01</t>
+          <t>IBKS01</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Tetragnatha_extensa</t>
+          <t>Rhomphaea_labiata</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -3178,28 +3206,28 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Theridiidae</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>2164</v>
+        <v>2249</v>
       </c>
       <c r="E90" t="n">
-        <v>484</v>
+        <v>427</v>
       </c>
       <c r="F90" t="n">
-        <v>2648</v>
+        <v>2676</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>IAHF01</t>
+          <t>ICFA01</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Tetragnatha_filiciphilia</t>
+          <t>Theridion_varians</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -3209,28 +3237,28 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Theridiidae</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>2257</v>
+        <v>2235</v>
       </c>
       <c r="E91" t="n">
-        <v>499</v>
+        <v>417</v>
       </c>
       <c r="F91" t="n">
-        <v>2756</v>
+        <v>2652</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>GITN01</t>
+          <t>ICEL01</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Tetragnatha_mandibulata</t>
+          <t>Argyrodes_miniaceus</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -3240,28 +3268,28 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Theridiidae</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>2231</v>
+        <v>2226</v>
       </c>
       <c r="E92" t="n">
-        <v>470</v>
+        <v>417</v>
       </c>
       <c r="F92" t="n">
-        <v>2701</v>
+        <v>2643</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>ICFC01</t>
+          <t>IBQT01</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Tetragnatha_maxillosa</t>
+          <t>Chrysso_octomaculata</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3271,28 +3299,28 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Theridiidae</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>2199</v>
+        <v>2212</v>
       </c>
       <c r="E93" t="n">
-        <v>448</v>
+        <v>537</v>
       </c>
       <c r="F93" t="n">
-        <v>2647</v>
+        <v>2749</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>ICMP01</t>
+          <t>IBWR01</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Tetragnatha_paludicola</t>
+          <t>Parasteatoda_culicivora</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -3302,28 +3330,28 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Theridiidae</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>2260</v>
+        <v>2204</v>
       </c>
       <c r="E94" t="n">
-        <v>544</v>
+        <v>439</v>
       </c>
       <c r="F94" t="n">
-        <v>2804</v>
+        <v>2643</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>GITO01</t>
+          <t>IBTW01</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Tetragnatha_quasimodo</t>
+          <t>Lehtinelagia_evanida</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -3333,28 +3361,28 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Thomisidae</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>2258</v>
+        <v>2319</v>
       </c>
       <c r="E95" t="n">
-        <v>534</v>
+        <v>324</v>
       </c>
       <c r="F95" t="n">
-        <v>2792</v>
+        <v>2643</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>GITP01</t>
+          <t>IBFM01</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Tetragnatha_stelarobusta</t>
+          <t>Diaea_subdola</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3364,28 +3392,28 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Thomisidae</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>2226</v>
+        <v>2281</v>
       </c>
       <c r="E96" t="n">
-        <v>565</v>
+        <v>416</v>
       </c>
       <c r="F96" t="n">
-        <v>2791</v>
+        <v>2697</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>GITQ01</t>
+          <t>ICGF01</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Tetragnatha_vermiformis</t>
+          <t>Pharta_brevipalpus</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3395,28 +3423,28 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Thomisidae</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>2267</v>
+        <v>2281</v>
       </c>
       <c r="E97" t="n">
-        <v>374</v>
+        <v>388</v>
       </c>
       <c r="F97" t="n">
-        <v>2641</v>
+        <v>2669</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>IAJJ01</t>
+          <t>IAWA01</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Tetragnatha_waikamoi</t>
+          <t>Ebrechtella_tricuspidata</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3426,28 +3454,28 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Thomisidae</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>2266</v>
+        <v>2256</v>
       </c>
       <c r="E98" t="n">
-        <v>527</v>
+        <v>389</v>
       </c>
       <c r="F98" t="n">
-        <v>2793</v>
+        <v>2645</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>GITR01</t>
+          <t>ICBZ01</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Tetragnatha_yesoensis</t>
+          <t>Oxytate_striatipes</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3457,28 +3485,28 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Tetragnathidae</t>
+          <t>Thomisidae</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>2184</v>
+        <v>2242</v>
       </c>
       <c r="E99" t="n">
-        <v>508</v>
+        <v>483</v>
       </c>
       <c r="F99" t="n">
-        <v>2692</v>
+        <v>2725</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>IBMZ01, DRR297344</t>
+          <t>IALM01</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Theridion_varians</t>
+          <t>Stephanopis_cambridgei</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3488,28 +3516,28 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Theridiidae</t>
+          <t>Thomisidae</t>
         </is>
       </c>
       <c r="D100" t="n">
         <v>2235</v>
       </c>
       <c r="E100" t="n">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="F100" t="n">
-        <v>2652</v>
+        <v>2651</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>ICEL01</t>
+          <t>ICHM01</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Uloborus_diversus</t>
+          <t>Ozyptila_nongae</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3519,28 +3547,28 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Uloboridae</t>
+          <t>Thomisidae</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>2137</v>
+        <v>2177</v>
       </c>
       <c r="E101" t="n">
-        <v>743</v>
+        <v>536</v>
       </c>
       <c r="F101" t="n">
-        <v>2880</v>
+        <v>2713</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>GJZJ01</t>
+          <t>ICBR01</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Ummeliata_osakaensis</t>
+          <t>Uloborus_diversus</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -3550,48 +3578,52 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Linyphiidae</t>
+          <t>Uloboridae</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>2214</v>
+        <v>2137</v>
       </c>
       <c r="E102" t="n">
-        <v>552</v>
+        <v>743</v>
       </c>
       <c r="F102" t="n">
-        <v>2766</v>
-      </c>
-      <c r="G102" t="inlineStr"/>
+        <v>2880</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>GJZJ01</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Zelotes_iriomotensis</t>
+          <t>Antrodiaetus_roretzi</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Araneomorphae</t>
+          <t>Mygalomorphae</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Gnaphosidae</t>
+          <t>Antrodiaetidae</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>2214</v>
+        <v>2190</v>
       </c>
       <c r="E103" t="n">
-        <v>514</v>
+        <v>349</v>
       </c>
       <c r="F103" t="n">
-        <v>2728</v>
+        <v>2539</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>IAHP01</t>
+          <t>IBPI01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update tables with udiv blast hits; revert parser
</commit_message>
<xml_diff>
--- a/results/Supplementary_Table_1_SpiderAccessions_BUSCOs.xlsx
+++ b/results/Supplementary_Table_1_SpiderAccessions_BUSCOs.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,37 +429,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Species</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Infraorder</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Family</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Single_copy_BUSCOs</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Duplicated_BUSCOs</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Total_BUSCOs</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Accession</t>
         </is>

</xml_diff>